<commit_message>
Deploy The Monolith Dashboard
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -472,21 +472,21 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
+        <v>370</v>
       </c>
       <c r="E2" t="n">
-        <v>145</v>
+        <v>93.31999999999999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -495,21 +495,21 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E3" t="n">
-        <v>350</v>
+        <v>147.19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -518,16 +518,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="E4" t="n">
-        <v>280</v>
+        <v>193.89</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -541,21 +541,21 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>60</v>
+        <v>131</v>
       </c>
       <c r="E5" t="n">
-        <v>180</v>
+        <v>66.86</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -564,21 +564,21 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>40</v>
+        <v>137</v>
       </c>
       <c r="E6" t="n">
-        <v>130</v>
+        <v>264.06</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -587,33 +587,631 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>25</v>
+        <v>313</v>
       </c>
       <c r="E7" t="n">
-        <v>120</v>
+        <v>186.55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>107</v>
+      </c>
+      <c r="E8" t="n">
+        <v>214.71</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>348</v>
+      </c>
+      <c r="E9" t="n">
+        <v>189.13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>118</v>
+      </c>
+      <c r="E10" t="n">
+        <v>331.29</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>282</v>
+      </c>
+      <c r="E11" t="n">
+        <v>426.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>250</v>
+      </c>
+      <c r="E12" t="n">
+        <v>177.42</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>195</v>
+      </c>
+      <c r="E13" t="n">
+        <v>294.92</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>490</v>
+      </c>
+      <c r="E14" t="n">
+        <v>395.22</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>117</v>
+      </c>
+      <c r="E15" t="n">
+        <v>66.08</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>WFC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>492</v>
+      </c>
+      <c r="E16" t="n">
+        <v>285.2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>434</v>
+      </c>
+      <c r="E17" t="n">
+        <v>99.67</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>327</v>
+      </c>
+      <c r="E18" t="n">
+        <v>204.96</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BLK</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>265</v>
+      </c>
+      <c r="E19" t="n">
+        <v>174.84</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>430</v>
+      </c>
+      <c r="E20" t="n">
+        <v>230.66</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>96</v>
+      </c>
+      <c r="E21" t="n">
+        <v>91.86</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>47</v>
+      </c>
+      <c r="E22" t="n">
+        <v>450.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>191</v>
+      </c>
+      <c r="E23" t="n">
+        <v>365.84</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MCD</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>89</v>
+      </c>
+      <c r="E24" t="n">
+        <v>352.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>264</v>
+      </c>
+      <c r="E25" t="n">
+        <v>291.96</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>157</v>
+      </c>
+      <c r="E26" t="n">
+        <v>85.89</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>52</v>
+      </c>
+      <c r="E27" t="n">
+        <v>95.02</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>383</v>
+      </c>
+      <c r="E28" t="n">
+        <v>339.58</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>BTC-USD</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Buy</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E8" t="n">
-        <v>30000</v>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>190</v>
+      </c>
+      <c r="E29" t="n">
+        <v>46360.28</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ETH-USD</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>130</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2916.03</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SOL-USD</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>103</v>
+      </c>
+      <c r="E31" t="n">
+        <v>61.13</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>122</v>
+      </c>
+      <c r="E32" t="n">
+        <v>95.23</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>CVX</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>359</v>
+      </c>
+      <c r="E33" t="n">
+        <v>284.78</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>121</v>
+      </c>
+      <c r="E34" t="n">
+        <v>369.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>